<commit_message>
dag & undirected shortest paths
</commit_message>
<xml_diff>
--- a/DSA_REV.xlsx
+++ b/DSA_REV.xlsx
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="106">
   <si>
     <t>problem</t>
   </si>
@@ -366,6 +366,18 @@
   </si>
   <si>
     <t>11may</t>
+  </si>
+  <si>
+    <t>802. Find Eventual Safe States</t>
+  </si>
+  <si>
+    <t>20may</t>
+  </si>
+  <si>
+    <t>542. 01 Matrix</t>
+  </si>
+  <si>
+    <t>21may</t>
   </si>
 </sst>
 </file>
@@ -1065,7 +1077,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1164,6 +1176,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1699,7 +1714,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AG44"/>
+  <dimension ref="A1:AG46"/>
   <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="8.81818181818182"/>
@@ -2233,11 +2248,14 @@
       </c>
     </row>
     <row r="24" ht="208" spans="1:33">
-      <c r="A24" s="9" t="s">
+      <c r="A24" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="B24" s="10">
+      <c r="B24" s="2">
         <v>46054</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="U24" s="25" t="s">
         <v>56</v>
@@ -2250,11 +2268,14 @@
       </c>
     </row>
     <row r="25" ht="156" spans="1:33">
-      <c r="A25" s="9" t="s">
+      <c r="A25" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="B25" s="10">
+      <c r="B25" s="21">
         <v>46054</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>6</v>
       </c>
       <c r="U25" s="8" t="s">
         <v>58</v>
@@ -2327,12 +2348,19 @@
       <c r="C28" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="U28" t="s">
+      <c r="U28" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="W28" s="10">
+      <c r="V28" s="1"/>
+      <c r="W28" s="2">
         <v>46083</v>
       </c>
+      <c r="X28" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="Y28" s="1"/>
+      <c r="Z28" s="1"/>
+      <c r="AA28" s="1"/>
     </row>
     <row r="29" ht="26" spans="1:33">
       <c r="A29" s="16" t="s">
@@ -2398,11 +2426,18 @@
       <c r="C31" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="U31" s="16" t="s">
+      <c r="U31" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="Z31" t="s">
+      <c r="V31" s="1"/>
+      <c r="W31" s="1"/>
+      <c r="X31" s="1"/>
+      <c r="Y31" s="1"/>
+      <c r="Z31" s="1" t="s">
         <v>75</v>
+      </c>
+      <c r="AA31" s="1" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="32" ht="260" spans="1:33">
@@ -2594,6 +2629,22 @@
       </c>
       <c r="E44" t="s">
         <v>101</v>
+      </c>
+    </row>
+    <row r="45" ht="26" spans="1:29">
+      <c r="A45" s="16" t="s">
+        <v>102</v>
+      </c>
+      <c r="F45" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="46" ht="26" spans="1:29">
+      <c r="A46" s="30" t="s">
+        <v>104</v>
+      </c>
+      <c r="D46" t="s">
+        <v>105</v>
       </c>
     </row>
   </sheetData>
@@ -2646,6 +2697,8 @@
     <hyperlink ref="A43" r:id="rId47" display="547. Number of Provinces" tooltip="https://leetcode.com/problems/number-of-provinces/"/>
     <hyperlink ref="A44" r:id="rId48" display="994. Rotting Oranges" tooltip="https://leetcode.com/problems/rotting-oranges/"/>
     <hyperlink ref="U37" r:id="rId49" display="1838. Frequency of the Most Frequent Element" tooltip="https://leetcode.com/problems/frequency-of-the-most-frequent-element/"/>
+    <hyperlink ref="A45" r:id="rId50" display="802. Find Eventual Safe States" tooltip="https://leetcode.com/problems/find-eventual-safe-states/"/>
+    <hyperlink ref="A46" r:id="rId51" display="542. 01 Matrix" tooltip="https://leetcode.com/problems/01-matrix/"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>

<commit_message>
bellman ford and floyd warshall algo
</commit_message>
<xml_diff>
--- a/DSA_REV.xlsx
+++ b/DSA_REV.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="18350" windowHeight="8000"/>
+    <workbookView windowWidth="18350" windowHeight="7400"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="110">
   <si>
     <t>problem</t>
   </si>
@@ -384,6 +384,12 @@
   </si>
   <si>
     <t>25may</t>
+  </si>
+  <si>
+    <t>787. Cheapest Flights Within K Stops</t>
+  </si>
+  <si>
+    <t>26may</t>
   </si>
 </sst>
 </file>
@@ -604,12 +610,12 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="9"/>
       <name val="Times New Roman"/>
       <charset val="0"/>
     </font>
     <font>
-      <b/>
       <sz val="9"/>
       <name val="Times New Roman"/>
       <charset val="0"/>
@@ -1184,8 +1190,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1720,7 +1726,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AG47"/>
+  <dimension ref="A1:AG48"/>
   <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="8.81818181818182"/>
@@ -2654,11 +2660,19 @@
       </c>
     </row>
     <row r="47" ht="156" spans="1:29">
-      <c r="A47" s="30" t="s">
+      <c r="A47" s="27" t="s">
         <v>106</v>
       </c>
       <c r="B47" t="s">
         <v>107</v>
+      </c>
+    </row>
+    <row r="48" ht="26" spans="1:29">
+      <c r="A48" s="30" t="s">
+        <v>108</v>
+      </c>
+      <c r="G48" t="s">
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -2714,6 +2728,7 @@
     <hyperlink ref="A45" r:id="rId50" display="802. Find Eventual Safe States" tooltip="https://leetcode.com/problems/find-eventual-safe-states/"/>
     <hyperlink ref="A46" r:id="rId51" display="542. 01 Matrix" tooltip="https://leetcode.com/problems/01-matrix/"/>
     <hyperlink ref="A47" r:id="rId52" display="1631. Path With Minimum Effort" tooltip="https://leetcode.com/problems/path-with-minimum-effort/"/>
+    <hyperlink ref="A48" r:id="rId53" display="787. Cheapest Flights Within K Stops" tooltip="https://leetcode.com/problems/cheapest-flights-within-k-stops/"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>